<commit_message>
Reports auto update (member)
</commit_message>
<xml_diff>
--- a/reports/member_funnel/downloads/member_funnel_1y_target_segments.xlsx
+++ b/reports/member_funnel/downloads/member_funnel_1y_target_segments.xlsx
@@ -5387,12 +5387,12 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>fkilove</t>
+          <t>ace1331</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>01080118915</t>
+          <t>01033906903</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -5402,7 +5402,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>bizboard</t>
+          <t>EDM_0502</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
@@ -5415,12 +5415,12 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ace1331</t>
+          <t>fkilove</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>01033906903</t>
+          <t>01080118915</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>EDM_0502</t>
+          <t>bizboard</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -7151,22 +7151,22 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>kk_5009517640</t>
+          <t>kk_2770056564</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>01090817520</t>
+          <t>01097609451</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>방문_하이브리드 오디언스</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
       <c r="E241" t="inlineStr"/>
@@ -7179,22 +7179,22 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>kk_2770056564</t>
+          <t>kk_5009517640</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>01097609451</t>
+          <t>01090817520</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>KAKAO_CH_event</t>
+          <t>방문_하이브리드 오디언스</t>
         </is>
       </c>
       <c r="E242" t="inlineStr"/>
@@ -12331,12 +12331,12 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>kk_4611877390</t>
+          <t>kk_3440880252</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>01034010575</t>
+          <t>01023828239</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -12346,7 +12346,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>demendgen</t>
+          <t>(referral)</t>
         </is>
       </c>
       <c r="E426" t="inlineStr"/>
@@ -12359,12 +12359,12 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>kk_3440880252</t>
+          <t>kk_4611877390</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>01023828239</t>
+          <t>01034010575</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>(referral)</t>
+          <t>demendgen</t>
         </is>
       </c>
       <c r="E427" t="inlineStr"/>
@@ -12751,22 +12751,22 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>kk_3181390163</t>
+          <t>kk_4486967764</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>01081430435</t>
+          <t>01095303556</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Organic Traffic</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>KAKAO_CH_event</t>
+          <t>(organic)</t>
         </is>
       </c>
       <c r="E441" t="inlineStr"/>
@@ -12779,22 +12779,22 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>kk_4486967764</t>
+          <t>kk_3181390163</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>01095303556</t>
+          <t>01081430435</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Organic Traffic</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>(organic)</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
       <c r="E442" t="inlineStr"/>
@@ -13507,12 +13507,12 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>kk_3866704464</t>
+          <t>kk_3377297415</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>01096848789</t>
+          <t>01088479524</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
@@ -13522,7 +13522,7 @@
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>KAKAO_alimtalk</t>
         </is>
       </c>
       <c r="E468" t="inlineStr"/>
@@ -13535,12 +13535,12 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>kk_3377297415</t>
+          <t>kk_3866704464</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>01088479524</t>
+          <t>01096848789</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
@@ -13550,7 +13550,7 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>KAKAO_alimtalk</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E469" t="inlineStr"/>
@@ -15635,12 +15635,12 @@
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>youl29</t>
+          <t>kk_4602095632</t>
         </is>
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>01050134121</t>
+          <t>01033213747</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
@@ -15663,12 +15663,12 @@
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>kk_4602095632</t>
+          <t>youl29</t>
         </is>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>01033213747</t>
+          <t>01050134121</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
@@ -16447,12 +16447,12 @@
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>pjh5540</t>
+          <t>kk_4912807536</t>
         </is>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>01085559978</t>
+          <t>01046055617</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
@@ -16462,7 +16462,7 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>KAKAO_CH_event</t>
+          <t>gdn</t>
         </is>
       </c>
       <c r="E573" t="inlineStr"/>
@@ -16475,12 +16475,12 @@
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>kk_4912807536</t>
+          <t>pjh5540</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>01046055617</t>
+          <t>01085559978</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
@@ -16490,7 +16490,7 @@
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>gdn</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
       <c r="E574" t="inlineStr"/>
@@ -18099,22 +18099,22 @@
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>kk_4705329623</t>
+          <t>jk571957</t>
         </is>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>01064926793</t>
+          <t>01080011083</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Organic Traffic</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>Organic Traffic</t>
         </is>
       </c>
       <c r="E632" t="inlineStr"/>
@@ -18155,22 +18155,22 @@
     <row r="634">
       <c r="A634" t="inlineStr">
         <is>
-          <t>jk571957</t>
+          <t>kk_4705329623</t>
         </is>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>01080011083</t>
+          <t>01064926793</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>Organic Traffic</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="D634" t="inlineStr">
         <is>
-          <t>Organic Traffic</t>
+          <t>LMS_ECOM_0214_newyear</t>
         </is>
       </c>
       <c r="E634" t="inlineStr"/>
@@ -19751,12 +19751,12 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>kk_4318436675</t>
+          <t>kk_3786745879</t>
         </is>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>01031176390</t>
+          <t>01093675013</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
@@ -19766,7 +19766,7 @@
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>KAKAO_CH_event</t>
+          <t>LMS_ECOM_0214_newyear</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
@@ -19779,12 +19779,12 @@
     <row r="692">
       <c r="A692" t="inlineStr">
         <is>
-          <t>kk_3786745879</t>
+          <t>kk_4318436675</t>
         </is>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>01093675013</t>
+          <t>01031176390</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
@@ -19794,7 +19794,7 @@
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
       <c r="E692" t="inlineStr"/>
@@ -19947,12 +19947,12 @@
     <row r="698">
       <c r="A698" t="inlineStr">
         <is>
-          <t>nikemkr</t>
+          <t>kk_4725433749</t>
         </is>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>01032361592</t>
+          <t>01096687926</t>
         </is>
       </c>
       <c r="C698" t="inlineStr">
@@ -19962,7 +19962,7 @@
       </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>naver_brandsearch_mobile</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="E698" t="inlineStr"/>
@@ -19975,12 +19975,12 @@
     <row r="699">
       <c r="A699" t="inlineStr">
         <is>
-          <t>kk_4725433749</t>
+          <t>nikemkr</t>
         </is>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>01096687926</t>
+          <t>01032361592</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
@@ -19990,7 +19990,7 @@
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>naver_brandsearch_mobile</t>
         </is>
       </c>
       <c r="E699" t="inlineStr"/>
@@ -20003,12 +20003,12 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>kk_4455109384</t>
+          <t>kk_3911965677</t>
         </is>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>01025222519</t>
+          <t>01029276124</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
@@ -20031,12 +20031,12 @@
     <row r="701">
       <c r="A701" t="inlineStr">
         <is>
-          <t>kk_3911965677</t>
+          <t>kk_4455109384</t>
         </is>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>01029276124</t>
+          <t>01025222519</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
@@ -22103,22 +22103,22 @@
     <row r="775">
       <c r="A775" t="inlineStr">
         <is>
-          <t>kk_4857948457</t>
+          <t>lovelybeib</t>
         </is>
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>01058380760</t>
+          <t>01040981902</t>
         </is>
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D775" t="inlineStr">
         <is>
-          <t>컬럼비아_DPA_240530</t>
+          <t>미분류</t>
         </is>
       </c>
       <c r="E775" t="inlineStr"/>
@@ -22131,22 +22131,22 @@
     <row r="776">
       <c r="A776" t="inlineStr">
         <is>
-          <t>lovelybeib</t>
+          <t>kk_4857948457</t>
         </is>
       </c>
       <c r="B776" t="inlineStr">
         <is>
-          <t>01040981902</t>
+          <t>01058380760</t>
         </is>
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="D776" t="inlineStr">
         <is>
-          <t>미분류</t>
+          <t>컬럼비아_DPA_240530</t>
         </is>
       </c>
       <c r="E776" t="inlineStr"/>
@@ -22411,12 +22411,12 @@
     <row r="786">
       <c r="A786" t="inlineStr">
         <is>
-          <t>sephira</t>
+          <t>jokowoo</t>
         </is>
       </c>
       <c r="B786" t="inlineStr">
         <is>
-          <t>01041867593</t>
+          <t>01040299924</t>
         </is>
       </c>
       <c r="C786" t="inlineStr">
@@ -22426,7 +22426,7 @@
       </c>
       <c r="D786" t="inlineStr">
         <is>
-          <t>KAKAO_CH_event</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="E786" t="inlineStr"/>
@@ -22439,12 +22439,12 @@
     <row r="787">
       <c r="A787" t="inlineStr">
         <is>
-          <t>jokowoo</t>
+          <t>sephira</t>
         </is>
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>01040299924</t>
+          <t>01041867593</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
@@ -22454,7 +22454,7 @@
       </c>
       <c r="D787" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>KAKAO_CH_event</t>
         </is>
       </c>
       <c r="E787" t="inlineStr"/>
@@ -23615,12 +23615,12 @@
     <row r="829">
       <c r="A829" t="inlineStr">
         <is>
-          <t>kk_3179837389</t>
+          <t>kk_4582648301</t>
         </is>
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>01089490421</t>
+          <t>01040451815</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
@@ -23630,7 +23630,7 @@
       </c>
       <c r="D829" t="inlineStr">
         <is>
-          <t>0803_SUMMER_LAST_CHANCE</t>
+          <t>KAKAO_alimtalk</t>
         </is>
       </c>
       <c r="E829" t="inlineStr"/>
@@ -23643,12 +23643,12 @@
     <row r="830">
       <c r="A830" t="inlineStr">
         <is>
-          <t>kk_4582648301</t>
+          <t>kk_3179837389</t>
         </is>
       </c>
       <c r="B830" t="inlineStr">
         <is>
-          <t>01040451815</t>
+          <t>01089490421</t>
         </is>
       </c>
       <c r="C830" t="inlineStr">
@@ -23658,7 +23658,7 @@
       </c>
       <c r="D830" t="inlineStr">
         <is>
-          <t>KAKAO_alimtalk</t>
+          <t>0803_SUMMER_LAST_CHANCE</t>
         </is>
       </c>
       <c r="E830" t="inlineStr"/>
@@ -23783,12 +23783,12 @@
     <row r="835">
       <c r="A835" t="inlineStr">
         <is>
-          <t>kk_4604844467</t>
+          <t>kk_3750120343</t>
         </is>
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>01045678553</t>
+          <t>01092908890</t>
         </is>
       </c>
       <c r="C835" t="inlineStr">
@@ -23798,7 +23798,7 @@
       </c>
       <c r="D835" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>LMS_ECOM_0410exclusive2</t>
         </is>
       </c>
       <c r="E835" t="inlineStr"/>
@@ -23811,12 +23811,12 @@
     <row r="836">
       <c r="A836" t="inlineStr">
         <is>
-          <t>kk_3750120343</t>
+          <t>kk_4604844467</t>
         </is>
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>01092908890</t>
+          <t>01045678553</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
@@ -23826,7 +23826,7 @@
       </c>
       <c r="D836" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0410exclusive2</t>
+          <t>LMS_ECOM_0214_newyear</t>
         </is>
       </c>
       <c r="E836" t="inlineStr"/>
@@ -24119,22 +24119,22 @@
     <row r="847">
       <c r="A847" t="inlineStr">
         <is>
-          <t>kk_4298043202</t>
+          <t>tesung1133</t>
         </is>
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>01047114486</t>
+          <t>01080018889</t>
         </is>
       </c>
       <c r="C847" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="D847" t="inlineStr">
         <is>
-          <t>KAKAO_CH_MESSAGE_0226_GOODBYEWINTER</t>
+          <t>LMS_ECOM_200416_family</t>
         </is>
       </c>
       <c r="E847" t="inlineStr"/>
@@ -24147,22 +24147,22 @@
     <row r="848">
       <c r="A848" t="inlineStr">
         <is>
-          <t>tesung1133</t>
+          <t>kk_4298043202</t>
         </is>
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>01080018889</t>
+          <t>01047114486</t>
         </is>
       </c>
       <c r="C848" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="D848" t="inlineStr">
         <is>
-          <t>LMS_ECOM_200416_family</t>
+          <t>KAKAO_CH_MESSAGE_0226_GOODBYEWINTER</t>
         </is>
       </c>
       <c r="E848" t="inlineStr"/>
@@ -24371,12 +24371,12 @@
     <row r="856">
       <c r="A856" t="inlineStr">
         <is>
-          <t>kk_4354536465</t>
+          <t>leecs11124</t>
         </is>
       </c>
       <c r="B856" t="inlineStr">
         <is>
-          <t>01090782401</t>
+          <t>01037870639</t>
         </is>
       </c>
       <c r="C856" t="inlineStr">
@@ -24386,7 +24386,7 @@
       </c>
       <c r="D856" t="inlineStr">
         <is>
-          <t>KAKAO_alimtalk</t>
+          <t>EDM_0214</t>
         </is>
       </c>
       <c r="E856" t="inlineStr"/>
@@ -24399,12 +24399,12 @@
     <row r="857">
       <c r="A857" t="inlineStr">
         <is>
-          <t>leecs11124</t>
+          <t>kk_4354536465</t>
         </is>
       </c>
       <c r="B857" t="inlineStr">
         <is>
-          <t>01037870639</t>
+          <t>01090782401</t>
         </is>
       </c>
       <c r="C857" t="inlineStr">
@@ -24414,7 +24414,7 @@
       </c>
       <c r="D857" t="inlineStr">
         <is>
-          <t>EDM_0214</t>
+          <t>KAKAO_alimtalk</t>
         </is>
       </c>
       <c r="E857" t="inlineStr"/>
@@ -24707,12 +24707,12 @@
     <row r="868">
       <c r="A868" t="inlineStr">
         <is>
-          <t>kk_3809928726</t>
+          <t>kk_3166693744</t>
         </is>
       </c>
       <c r="B868" t="inlineStr">
         <is>
-          <t>01079193871</t>
+          <t>01045579380</t>
         </is>
       </c>
       <c r="C868" t="inlineStr">
@@ -24735,12 +24735,12 @@
     <row r="869">
       <c r="A869" t="inlineStr">
         <is>
-          <t>kk_3166693744</t>
+          <t>kk_3809928726</t>
         </is>
       </c>
       <c r="B869" t="inlineStr">
         <is>
-          <t>01045579380</t>
+          <t>01079193871</t>
         </is>
       </c>
       <c r="C869" t="inlineStr">
@@ -25239,12 +25239,12 @@
     <row r="887">
       <c r="A887" t="inlineStr">
         <is>
-          <t>kk_4864045300</t>
+          <t>kk_4376700680</t>
         </is>
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>01089985309</t>
+          <t>01047096832</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
@@ -25254,7 +25254,7 @@
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>[PF]전환_회원가입(유사)</t>
+          <t>LMS_ECOM_0425_FAMILYSALE</t>
         </is>
       </c>
       <c r="E887" t="inlineStr"/>
@@ -25267,12 +25267,12 @@
     <row r="888">
       <c r="A888" t="inlineStr">
         <is>
-          <t>kk_4376700680</t>
+          <t>kk_4864045300</t>
         </is>
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>01047096832</t>
+          <t>01089985309</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
@@ -25282,7 +25282,7 @@
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0425_FAMILYSALE</t>
+          <t>[PF]전환_회원가입(유사)</t>
         </is>
       </c>
       <c r="E888" t="inlineStr"/>
@@ -25491,22 +25491,22 @@
     <row r="896">
       <c r="A896" t="inlineStr">
         <is>
-          <t>kk_4977819786</t>
+          <t>kk_4286220576</t>
         </is>
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>01063257991</t>
+          <t>01053587782</t>
         </is>
       </c>
       <c r="C896" t="inlineStr">
         <is>
-          <t>Paid Ad</t>
+          <t>Owned Channel</t>
         </is>
       </c>
       <c r="D896" t="inlineStr">
         <is>
-          <t>naver_brandsearch_mobile</t>
+          <t>LMS_ECOM_200416_seasonoff</t>
         </is>
       </c>
       <c r="E896" t="inlineStr"/>
@@ -25519,22 +25519,22 @@
     <row r="897">
       <c r="A897" t="inlineStr">
         <is>
-          <t>kk_4286220576</t>
+          <t>kk_4977819786</t>
         </is>
       </c>
       <c r="B897" t="inlineStr">
         <is>
-          <t>01053587782</t>
+          <t>01063257991</t>
         </is>
       </c>
       <c r="C897" t="inlineStr">
         <is>
-          <t>Owned Channel</t>
+          <t>Paid Ad</t>
         </is>
       </c>
       <c r="D897" t="inlineStr">
         <is>
-          <t>LMS_ECOM_200416_seasonoff</t>
+          <t>naver_brandsearch_mobile</t>
         </is>
       </c>
       <c r="E897" t="inlineStr"/>
@@ -25631,12 +25631,12 @@
     <row r="901">
       <c r="A901" t="inlineStr">
         <is>
-          <t>kk_3957117484</t>
+          <t>khyoon99</t>
         </is>
       </c>
       <c r="B901" t="inlineStr">
         <is>
-          <t>01042204013</t>
+          <t>01044153686</t>
         </is>
       </c>
       <c r="C901" t="inlineStr">
@@ -25646,7 +25646,7 @@
       </c>
       <c r="D901" t="inlineStr">
         <is>
-          <t>0520</t>
+          <t>KAKAO_alimtalk</t>
         </is>
       </c>
       <c r="E901" t="inlineStr"/>
@@ -25659,12 +25659,12 @@
     <row r="902">
       <c r="A902" t="inlineStr">
         <is>
-          <t>kk_2825498802</t>
+          <t>kk_3957117484</t>
         </is>
       </c>
       <c r="B902" t="inlineStr">
         <is>
-          <t>01027817891</t>
+          <t>01042204013</t>
         </is>
       </c>
       <c r="C902" t="inlineStr">
@@ -25674,7 +25674,7 @@
       </c>
       <c r="D902" t="inlineStr">
         <is>
-          <t>LMS_ECOM_0214_newyear</t>
+          <t>0520</t>
         </is>
       </c>
       <c r="E902" t="inlineStr"/>
@@ -25687,12 +25687,12 @@
     <row r="903">
       <c r="A903" t="inlineStr">
         <is>
-          <t>jhj95</t>
+          <t>kk_2825498802</t>
         </is>
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>01031240827</t>
+          <t>01027817891</t>
         </is>
       </c>
       <c r="C903" t="inlineStr">
@@ -25702,7 +25702,7 @@
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>KAKAO_alimtalk</t>
+          <t>LMS_ECOM_0214_newyear</t>
         </is>
       </c>
       <c r="E903" t="inlineStr"/>
@@ -25715,12 +25715,12 @@
     <row r="904">
       <c r="A904" t="inlineStr">
         <is>
-          <t>khyoon99</t>
+          <t>jhj95</t>
         </is>
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>01044153686</t>
+          <t>01031240827</t>
         </is>
       </c>
       <c r="C904" t="inlineStr">

</xml_diff>